<commit_message>
Kundimporten läser Alternativa leveransadresser: adressens namn och Förvald
Leveransadressimporten mappar den upprepade Namn-kolumnen (adressens eget namn, sekundäralias) och den nya kolumnen Förvald, som avgör förvald adress per rad i stället för kryssrutan Sätt som förvald leveransadress. Manual, importmall, regelfil och tester (även mot den riktiga exporten) uppdaterade.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013pvWaFZiioxpDd9AVeYPCR
</commit_message>
<xml_diff>
--- a/apps/web/public/importmallar/importmall-kundadresser.xlsx
+++ b/apps/web/public/importmallar/importmall-kundadresser.xlsx
@@ -107,6 +107,18 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">Landskod med två bokstäver (t.ex. SE); små bokstäver godtas. Tom cell ger SE.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Ja/Nej, 1/0, X eller true/false — Ja gör adressen till kundens förvalda leveransadress. Är kolumnen med avgör den per rad i stället för kryssrutan Sätt som förvald leveransadress; har kunden redan en förvald adress blir det en varning och adressen läggs till utan att vara förvald.</t>
         </r>
       </text>
     </comment>
@@ -178,6 +190,7 @@
     <col min="6" max="6" width="14" customWidth="1" style="4"/>
     <col min="7" max="7" width="14" customWidth="1"/>
     <col min="8" max="8" width="14" customWidth="1"/>
+    <col min="9" max="9" width="14" customWidth="1" style="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -219,6 +232,11 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Land</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Förvald</t>
         </is>
       </c>
     </row>
@@ -472,6 +490,28 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Förvald</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nej</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ja/Nej, 1/0, X eller true/false — Ja gör adressen till kundens förvalda leveransadress. Är kolumnen med avgör den per rad i stället för kryssrutan Sätt som förvald leveransadress; har kunden redan en förvald adress blir det en varning och adressen läggs till utan att vara förvald.</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nej</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>